<commit_message>
Deploying to gh-pages from @ NIH-NCPI/ncpi-fhir-ig-2@d89aecd19da6bbdef7f57e3ec8fb170e6028db2a 🚀
</commit_message>
<xml_diff>
--- a/StructureDefinition-SharedDataModelFile.xlsx
+++ b/StructureDefinition-SharedDataModelFile.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2025-08-26T23:53:55+00:00</t>
+    <t>2025-12-03T18:37:31+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -369,7 +369,7 @@
     <t>A human language.</t>
   </si>
   <si>
-    <t>http://hl7.org/fhir/ValueSet/languages</t>
+    <t>http://hl7.org/fhir/ValueSet/languages|4.0.1</t>
   </si>
   <si>
     <t>Resource.language</t>
@@ -571,7 +571,7 @@
     <t>What the purpose of a list is.</t>
   </si>
   <si>
-    <t>http://hl7.org/fhir/ValueSet/list-example-codes</t>
+    <t>http://hl7.org/fhir/ValueSet/list-example-codes|4.0.1</t>
   </si>
   <si>
     <t>List.code</t>
@@ -580,7 +580,7 @@
     <t>SharedDataModelFile.location.subject</t>
   </si>
   <si>
-    <t xml:space="preserve">Reference(Patient|Group|Device|Location)
+    <t xml:space="preserve">Reference(Patient|4.0.1|Group|4.0.1|Device|4.0.1|Location|4.0.1)
 </t>
   </si>
   <si>
@@ -602,7 +602,7 @@
     <t>SharedDataModelFile.location.encounter</t>
   </si>
   <si>
-    <t xml:space="preserve">Reference(Encounter)
+    <t xml:space="preserve">Reference(Encounter|4.0.1)
 </t>
   </si>
   <si>
@@ -644,7 +644,7 @@
 </t>
   </si>
   <si>
-    <t xml:space="preserve">Reference(Practitioner|PractitionerRole|Patient|Device)
+    <t xml:space="preserve">Reference(Practitioner|4.0.1|PractitionerRole|4.0.1|Patient|4.0.1|Device|4.0.1)
 </t>
   </si>
   <si>
@@ -681,7 +681,7 @@
     <t>What order applies to the items in a list.</t>
   </si>
   <si>
-    <t>http://hl7.org/fhir/ValueSet/list-order</t>
+    <t>http://hl7.org/fhir/ValueSet/list-order|4.0.1</t>
   </si>
   <si>
     <t>List.orderedBy</t>
@@ -782,7 +782,7 @@
     <t>Codes that provide further information about the reason and meaning of the item in the list.</t>
   </si>
   <si>
-    <t>http://hl7.org/fhir/ValueSet/list-item-flag</t>
+    <t>http://hl7.org/fhir/ValueSet/list-item-flag|4.0.1</t>
   </si>
   <si>
     <t>List.entry.flag</t>
@@ -835,7 +835,7 @@
     <t>SharedDataModelFile.location.entry.item</t>
   </si>
   <si>
-    <t xml:space="preserve">Reference(Resource)
+    <t xml:space="preserve">Reference(Resource|4.0.1)
 </t>
   </si>
   <si>
@@ -866,7 +866,7 @@
     <t>If a list is empty, why it is empty.</t>
   </si>
   <si>
-    <t>http://hl7.org/fhir/ValueSet/list-empty-reason</t>
+    <t>http://hl7.org/fhir/ValueSet/list-empty-reason|4.0.1</t>
   </si>
   <si>
     <t>List.emptyReason</t>
@@ -1326,7 +1326,7 @@
     <col min="8" max="8" width="13.953125" customWidth="true" bestFit="true"/>
     <col min="9" max="9" width="11.3671875" customWidth="true" bestFit="true"/>
     <col min="10" max="10" width="20.703125" customWidth="true" bestFit="true"/>
-    <col min="11" max="11" width="44.3046875" customWidth="true" bestFit="true"/>
+    <col min="11" max="11" width="62.41796875" customWidth="true" bestFit="true"/>
     <col min="12" max="12" width="100.703125" customWidth="true" bestFit="true"/>
     <col min="13" max="13" width="100.703125" customWidth="true" bestFit="true"/>
     <col min="14" max="14" width="100.703125" customWidth="true" bestFit="true"/>
@@ -1341,7 +1341,7 @@
     <col min="23" max="23" width="16.3203125" customWidth="true" bestFit="true"/>
     <col min="24" max="24" width="16.16796875" customWidth="true" bestFit="true"/>
     <col min="25" max="25" width="73.66015625" customWidth="true" bestFit="true"/>
-    <col min="26" max="26" width="37.33203125" customWidth="true" bestFit="true"/>
+    <col min="26" max="26" width="41.86328125" customWidth="true" bestFit="true"/>
     <col min="27" max="27" width="5.44140625" customWidth="true" bestFit="true"/>
     <col min="28" max="28" width="19.4765625" customWidth="true" bestFit="true"/>
     <col min="29" max="29" width="17.65625" customWidth="true" bestFit="true"/>

</xml_diff>